<commit_message>
Correct Lesson 5 word 18 to piece
</commit_message>
<xml_diff>
--- a/data/Lesson_1-5_英文單字_繁中注音_總表.xlsx
+++ b/data/Lesson_1-5_英文單字_繁中注音_總表.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overall" sheetId="1" r:id="R25b09116b9fd4a66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 1" sheetId="2" r:id="Rf5bc3dd7fa1c4ca8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 2" sheetId="3" r:id="R69b227545e564ca7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 3" sheetId="4" r:id="R3a21e45bede44ef7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 4" sheetId="5" r:id="R1f66d2dccc7f49e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 5" sheetId="6" r:id="Rbb2ad0bf30794549"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overall" sheetId="1" r:id="R009e74619737426e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 1" sheetId="2" r:id="R3daa85ee6573420e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 2" sheetId="3" r:id="R407bc2a489354f5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 3" sheetId="4" r:id="R762e03745ce043a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 4" sheetId="5" r:id="R585adc32c52043cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson 5" sheetId="6" r:id="Rc49cd7d5b83f44a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5359,13 +5359,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="C267" s="16" t="str">
-        <x:v>pie</x:v>
+        <x:v>piece</x:v>
       </x:c>
       <x:c r="D267" s="16" t="str">
-        <x:v>派、餡餅</x:v>
+        <x:v>一片、一塊</x:v>
       </x:c>
       <x:c r="E267" s="16" t="str">
-        <x:v>ㄆㄞˋ、ㄒㄧㄢˋ ㄅㄧㄥˇ</x:v>
+        <x:v>ㄧˊ ㄆㄧㄢˋ、ㄧˊ ㄎㄨㄞˋ</x:v>
       </x:c>
       <x:c r="F267" s="15" t="str"/>
     </x:row>
@@ -5507,7 +5507,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f917450610843af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10514ad0864b4e30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6708,7 +6708,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b042edbf53a4824"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9148584f4f94417"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7894,7 +7894,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e3bd0ebc9a642dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49c3758470ec4c41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8543,7 +8543,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5141a3025b04cbc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cac396d82414691"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9486,7 +9486,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54d353ac0204488b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1907bc760ee54871"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9796,13 +9796,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B22" s="16" t="str">
-        <x:v>pie</x:v>
+        <x:v>piece</x:v>
       </x:c>
       <x:c r="C22" s="16" t="str">
-        <x:v>派、餡餅</x:v>
+        <x:v>一片、一塊</x:v>
       </x:c>
       <x:c r="D22" s="16" t="str">
-        <x:v>ㄆㄞˋ、ㄒㄧㄢˋ ㄅㄧㄥˇ</x:v>
+        <x:v>ㄧˊ ㄆㄧㄢˋ、ㄧˊ ㄎㄨㄞˋ</x:v>
       </x:c>
       <x:c r="E22" s="15" t="str"/>
     </x:row>
@@ -9928,7 +9928,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d954f62b7af4f28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R716ab05fc5b34e85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>